<commit_message>
rerun model qwen3.5:9b RAG TOT Model results generated
</commit_message>
<xml_diff>
--- a/results/qwen3_5_9b/comparison_ToTRAG/ToTRAG_costs.xlsx
+++ b/results/qwen3_5_9b/comparison_ToTRAG/ToTRAG_costs.xlsx
@@ -472,25 +472,25 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>3.514173030853271</v>
+        <v>695.3608591556549</v>
       </c>
       <c r="B2" t="n">
-        <v>1420.859375</v>
+        <v>1424.546875</v>
       </c>
       <c r="C2" t="n">
-        <v>10.9</v>
+        <v>14.7</v>
       </c>
       <c r="D2" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>0.3115198612213135</v>
+        <v>0.6841831207275391</v>
       </c>
       <c r="G2" t="n">
-        <v>3.202648639678955</v>
+        <v>694.6766669750214</v>
       </c>
       <c r="H2" t="n">
         <v>0</v>
@@ -498,25 +498,25 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>6.709547281265259</v>
+        <v>531.6408832073212</v>
       </c>
       <c r="B3" t="n">
-        <v>1421.046875</v>
+        <v>1424.71875</v>
       </c>
       <c r="C3" t="n">
-        <v>9.4</v>
+        <v>14.8</v>
       </c>
       <c r="D3" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="E3" t="n">
         <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>0.05140066146850586</v>
+        <v>1.485445737838745</v>
       </c>
       <c r="G3" t="n">
-        <v>6.658143043518066</v>
+        <v>530.1554305553436</v>
       </c>
       <c r="H3" t="n">
         <v>0</v>
@@ -524,25 +524,25 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>5.542050123214722</v>
+        <v>505.5695912837982</v>
       </c>
       <c r="B4" t="n">
-        <v>1421.17578125</v>
+        <v>1424.77734375</v>
       </c>
       <c r="C4" t="n">
-        <v>14.1</v>
+        <v>14.7</v>
       </c>
       <c r="D4" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>0.05872344970703125</v>
+        <v>1.269025802612305</v>
       </c>
       <c r="G4" t="n">
-        <v>5.483324289321899</v>
+        <v>504.3005628585815</v>
       </c>
       <c r="H4" t="n">
         <v>0</v>
@@ -550,25 +550,25 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>2.96129584312439</v>
+        <v>654.1937582492828</v>
       </c>
       <c r="B5" t="n">
-        <v>1421.19921875</v>
+        <v>1427.05078125</v>
       </c>
       <c r="C5" t="n">
-        <v>9.199999999999999</v>
+        <v>14.8</v>
       </c>
       <c r="D5" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>0.05079221725463867</v>
+        <v>1.24380898475647</v>
       </c>
       <c r="G5" t="n">
-        <v>2.91050124168396</v>
+        <v>652.949946641922</v>
       </c>
       <c r="H5" t="n">
         <v>0</v>
@@ -576,25 +576,25 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>2.571090698242188</v>
+        <v>1096.280446767807</v>
       </c>
       <c r="B6" t="n">
-        <v>1421.28125</v>
+        <v>1429.56640625</v>
       </c>
       <c r="C6" t="n">
-        <v>9.1</v>
+        <v>14.9</v>
       </c>
       <c r="D6" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="E6" t="n">
         <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>0.04886579513549805</v>
+        <v>1.249656200408936</v>
       </c>
       <c r="G6" t="n">
-        <v>2.522222757339478</v>
+        <v>1095.030787944794</v>
       </c>
       <c r="H6" t="n">
         <v>0</v>
@@ -602,25 +602,25 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>4.446542501449585</v>
+        <v>1282.672055721283</v>
       </c>
       <c r="B7" t="n">
-        <v>1421.4375</v>
+        <v>1430.22265625</v>
       </c>
       <c r="C7" t="n">
-        <v>11.6</v>
+        <v>14.9</v>
       </c>
       <c r="D7" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="E7" t="n">
         <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>0.04900312423706055</v>
+        <v>1.275151014328003</v>
       </c>
       <c r="G7" t="n">
-        <v>4.397536993026733</v>
+        <v>1281.396900653839</v>
       </c>
       <c r="H7" t="n">
         <v>0</v>
@@ -628,25 +628,25 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>4.116216659545898</v>
+        <v>1184.164467811584</v>
       </c>
       <c r="B8" t="n">
-        <v>1421.58203125</v>
+        <v>1430.87109375</v>
       </c>
       <c r="C8" t="n">
-        <v>13.1</v>
+        <v>15</v>
       </c>
       <c r="D8" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="E8" t="n">
         <v>0</v>
       </c>
       <c r="F8" t="n">
-        <v>0.06111049652099609</v>
+        <v>1.25953197479248</v>
       </c>
       <c r="G8" t="n">
-        <v>4.055103302001953</v>
+        <v>1182.904933929443</v>
       </c>
       <c r="H8" t="n">
         <v>0</v>
@@ -654,25 +654,25 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>3.427034378051758</v>
+        <v>645.8816244602203</v>
       </c>
       <c r="B9" t="n">
-        <v>1421.62109375</v>
+        <v>1430.875</v>
       </c>
       <c r="C9" t="n">
-        <v>9.1</v>
+        <v>14.8</v>
       </c>
       <c r="D9" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="E9" t="n">
         <v>0</v>
       </c>
       <c r="F9" t="n">
-        <v>0.05016899108886719</v>
+        <v>1.274761438369751</v>
       </c>
       <c r="G9" t="n">
-        <v>3.376862287521362</v>
+        <v>644.6068601608276</v>
       </c>
       <c r="H9" t="n">
         <v>0</v>
@@ -680,25 +680,25 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>2.672636747360229</v>
+        <v>850.9556107521057</v>
       </c>
       <c r="B10" t="n">
-        <v>1421.625</v>
+        <v>1430.8828125</v>
       </c>
       <c r="C10" t="n">
-        <v>9.5</v>
+        <v>14.9</v>
       </c>
       <c r="D10" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="E10" t="n">
         <v>0</v>
       </c>
       <c r="F10" t="n">
-        <v>0.05249142646789551</v>
+        <v>1.289028644561768</v>
       </c>
       <c r="G10" t="n">
-        <v>2.620143175125122</v>
+        <v>849.6665790081024</v>
       </c>
       <c r="H10" t="n">
         <v>0</v>
@@ -706,25 +706,25 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>3.0864577293396</v>
+        <v>650.7179703712463</v>
       </c>
       <c r="B11" t="n">
-        <v>1421.64453125</v>
+        <v>1430.8828125</v>
       </c>
       <c r="C11" t="n">
-        <v>13.8</v>
+        <v>14.8</v>
       </c>
       <c r="D11" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="E11" t="n">
         <v>0</v>
       </c>
       <c r="F11" t="n">
-        <v>0.05005407333374023</v>
+        <v>1.241165399551392</v>
       </c>
       <c r="G11" t="n">
-        <v>3.036401033401489</v>
+        <v>649.4768023490906</v>
       </c>
       <c r="H11" t="n">
         <v>0</v>
@@ -732,25 +732,25 @@
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>6.718741416931152</v>
+        <v>610.5229642391205</v>
       </c>
       <c r="B12" t="n">
-        <v>1421.65625</v>
+        <v>1430.8828125</v>
       </c>
       <c r="C12" t="n">
-        <v>11.3</v>
+        <v>14.8</v>
       </c>
       <c r="D12" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="E12" t="n">
         <v>0</v>
       </c>
       <c r="F12" t="n">
-        <v>0.04909992218017578</v>
+        <v>1.235222816467285</v>
       </c>
       <c r="G12" t="n">
-        <v>6.669639110565186</v>
+        <v>609.2877380847931</v>
       </c>
       <c r="H12" t="n">
         <v>0</v>
@@ -758,25 +758,25 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>2.449448823928833</v>
+        <v>645.6885144710541</v>
       </c>
       <c r="B13" t="n">
-        <v>1421.6796875</v>
+        <v>1430.8828125</v>
       </c>
       <c r="C13" t="n">
-        <v>9.1</v>
+        <v>14.9</v>
       </c>
       <c r="D13" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="E13" t="n">
         <v>0</v>
       </c>
       <c r="F13" t="n">
-        <v>0.04813027381896973</v>
+        <v>1.22734522819519</v>
       </c>
       <c r="G13" t="n">
-        <v>2.401316165924072</v>
+        <v>644.4611659049988</v>
       </c>
       <c r="H13" t="n">
         <v>0</v>
@@ -784,25 +784,25 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>6.250750303268433</v>
+        <v>851.3273868560791</v>
       </c>
       <c r="B14" t="n">
-        <v>1421.74609375</v>
+        <v>1430.8828125</v>
       </c>
       <c r="C14" t="n">
-        <v>13.8</v>
+        <v>14.9</v>
       </c>
       <c r="D14" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="E14" t="n">
         <v>0</v>
       </c>
       <c r="F14" t="n">
-        <v>0.04938817024230957</v>
+        <v>1.242627382278442</v>
       </c>
       <c r="G14" t="n">
-        <v>6.201359510421753</v>
+        <v>850.0847568511963</v>
       </c>
       <c r="H14" t="n">
         <v>0</v>
@@ -810,25 +810,25 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>3.409560441970825</v>
+        <v>683.0590803623199</v>
       </c>
       <c r="B15" t="n">
-        <v>1421.74609375</v>
+        <v>1430.8828125</v>
       </c>
       <c r="C15" t="n">
-        <v>9.300000000000001</v>
+        <v>14.9</v>
       </c>
       <c r="D15" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="E15" t="n">
         <v>0</v>
       </c>
       <c r="F15" t="n">
-        <v>0.04938602447509766</v>
+        <v>1.301464796066284</v>
       </c>
       <c r="G15" t="n">
-        <v>3.360171556472778</v>
+        <v>681.7576134204865</v>
       </c>
       <c r="H15" t="n">
         <v>0</v>
@@ -836,25 +836,25 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>3.407259702682495</v>
+        <v>634.9633483886719</v>
       </c>
       <c r="B16" t="n">
-        <v>1421.74609375</v>
+        <v>1430.8828125</v>
       </c>
       <c r="C16" t="n">
-        <v>9</v>
+        <v>14.9</v>
       </c>
       <c r="D16" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="E16" t="n">
         <v>0</v>
       </c>
       <c r="F16" t="n">
-        <v>0.04798340797424316</v>
+        <v>1.272817850112915</v>
       </c>
       <c r="G16" t="n">
-        <v>3.35927414894104</v>
+        <v>633.6905281543732</v>
       </c>
       <c r="H16" t="n">
         <v>0</v>
@@ -862,25 +862,25 @@
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>5.538920164108276</v>
+        <v>870.301830291748</v>
       </c>
       <c r="B17" t="n">
-        <v>1421.8046875</v>
+        <v>1430.8828125</v>
       </c>
       <c r="C17" t="n">
-        <v>14.3</v>
+        <v>14.9</v>
       </c>
       <c r="D17" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="E17" t="n">
         <v>0</v>
       </c>
       <c r="F17" t="n">
-        <v>0.05006098747253418</v>
+        <v>1.228122234344482</v>
       </c>
       <c r="G17" t="n">
-        <v>5.488856792449951</v>
+        <v>869.0737059116364</v>
       </c>
       <c r="H17" t="n">
         <v>0</v>
@@ -888,25 +888,25 @@
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>5.91644024848938</v>
+        <v>726.078840970993</v>
       </c>
       <c r="B18" t="n">
-        <v>1421.83984375</v>
+        <v>1430.8828125</v>
       </c>
       <c r="C18" t="n">
-        <v>9.300000000000001</v>
+        <v>14.9</v>
       </c>
       <c r="D18" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="E18" t="n">
         <v>0</v>
       </c>
       <c r="F18" t="n">
-        <v>0.04915428161621094</v>
+        <v>1.268083095550537</v>
       </c>
       <c r="G18" t="n">
-        <v>5.86728310585022</v>
+        <v>724.8107545375824</v>
       </c>
       <c r="H18" t="n">
         <v>0</v>
@@ -914,25 +914,25 @@
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>3.519678354263306</v>
+        <v>769.8312909603119</v>
       </c>
       <c r="B19" t="n">
-        <v>1421.8828125</v>
+        <v>1430.8828125</v>
       </c>
       <c r="C19" t="n">
-        <v>9.1</v>
+        <v>14.9</v>
       </c>
       <c r="D19" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="E19" t="n">
         <v>0</v>
       </c>
       <c r="F19" t="n">
-        <v>0.04809069633483887</v>
+        <v>1.232758760452271</v>
       </c>
       <c r="G19" t="n">
-        <v>3.471585512161255</v>
+        <v>768.5985298156738</v>
       </c>
       <c r="H19" t="n">
         <v>0</v>
@@ -940,25 +940,25 @@
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>4.015764236450195</v>
+        <v>710.5408804416656</v>
       </c>
       <c r="B20" t="n">
-        <v>1421.9140625</v>
+        <v>1430.8828125</v>
       </c>
       <c r="C20" t="n">
-        <v>16</v>
+        <v>14.9</v>
       </c>
       <c r="D20" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="E20" t="n">
         <v>0</v>
       </c>
       <c r="F20" t="n">
-        <v>0.05057668685913086</v>
+        <v>1.257959127426147</v>
       </c>
       <c r="G20" t="n">
-        <v>3.965185165405273</v>
+        <v>709.2829184532166</v>
       </c>
       <c r="H20" t="n">
         <v>0</v>
@@ -966,25 +966,25 @@
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>10.57776641845703</v>
+        <v>3267.928041696548</v>
       </c>
       <c r="B21" t="n">
-        <v>1422.25</v>
+        <v>1437.8203125</v>
       </c>
       <c r="C21" t="n">
-        <v>10.5</v>
+        <v>15</v>
       </c>
       <c r="D21" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="E21" t="n">
         <v>0</v>
       </c>
       <c r="F21" t="n">
-        <v>0.0477144718170166</v>
+        <v>1.511253356933594</v>
       </c>
       <c r="G21" t="n">
-        <v>10.53004908561707</v>
+        <v>3266.416784763336</v>
       </c>
       <c r="H21" t="n">
         <v>0</v>
@@ -992,25 +992,25 @@
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>2.628326892852783</v>
+        <v>600.7188527584076</v>
       </c>
       <c r="B22" t="n">
-        <v>1422.3046875</v>
+        <v>1437.8203125</v>
       </c>
       <c r="C22" t="n">
-        <v>14.3</v>
+        <v>14.9</v>
       </c>
       <c r="D22" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="E22" t="n">
         <v>0</v>
       </c>
       <c r="F22" t="n">
-        <v>0.04940271377563477</v>
+        <v>1.461212158203125</v>
       </c>
       <c r="G22" t="n">
-        <v>2.578921556472778</v>
+        <v>599.2576377391815</v>
       </c>
       <c r="H22" t="n">
         <v>0</v>
@@ -1018,25 +1018,25 @@
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>3.166445732116699</v>
+        <v>1094.860126018524</v>
       </c>
       <c r="B23" t="n">
-        <v>1422.3125</v>
+        <v>1441.01171875</v>
       </c>
       <c r="C23" t="n">
-        <v>9.4</v>
+        <v>14.3</v>
       </c>
       <c r="D23" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="E23" t="n">
         <v>0</v>
       </c>
       <c r="F23" t="n">
-        <v>0.04829621315002441</v>
+        <v>0.7324140071868896</v>
       </c>
       <c r="G23" t="n">
-        <v>3.118146657943726</v>
+        <v>1094.127707958221</v>
       </c>
       <c r="H23" t="n">
         <v>0</v>
@@ -1044,25 +1044,25 @@
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>4.142622947692871</v>
+        <v>681.2412395477295</v>
       </c>
       <c r="B24" t="n">
-        <v>1422.3125</v>
+        <v>1441.0234375</v>
       </c>
       <c r="C24" t="n">
-        <v>9.1</v>
+        <v>14.8</v>
       </c>
       <c r="D24" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="E24" t="n">
         <v>0</v>
       </c>
       <c r="F24" t="n">
-        <v>0.05130624771118164</v>
+        <v>0.337653636932373</v>
       </c>
       <c r="G24" t="n">
-        <v>4.091314315795898</v>
+        <v>680.903582572937</v>
       </c>
       <c r="H24" t="n">
         <v>0</v>
@@ -1070,25 +1070,25 @@
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>4.561594247817993</v>
+        <v>739.4099335670471</v>
       </c>
       <c r="B25" t="n">
-        <v>1422.31640625</v>
+        <v>1441.4453125</v>
       </c>
       <c r="C25" t="n">
-        <v>15.2</v>
+        <v>15</v>
       </c>
       <c r="D25" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="E25" t="n">
         <v>0</v>
       </c>
       <c r="F25" t="n">
-        <v>0.0504915714263916</v>
+        <v>0.2949469089508057</v>
       </c>
       <c r="G25" t="n">
-        <v>4.511099815368652</v>
+        <v>739.1149845123291</v>
       </c>
       <c r="H25" t="n">
         <v>0</v>
@@ -1096,25 +1096,25 @@
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>2.947563409805298</v>
+        <v>556.9603869915009</v>
       </c>
       <c r="B26" t="n">
-        <v>1422.31640625</v>
+        <v>1442.5859375</v>
       </c>
       <c r="C26" t="n">
-        <v>9.4</v>
+        <v>14.8</v>
       </c>
       <c r="D26" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="E26" t="n">
         <v>0</v>
       </c>
       <c r="F26" t="n">
-        <v>0.05006122589111328</v>
+        <v>0.3099029064178467</v>
       </c>
       <c r="G26" t="n">
-        <v>2.897499799728394</v>
+        <v>556.6504819393158</v>
       </c>
       <c r="H26" t="n">
         <v>0</v>
@@ -1122,25 +1122,25 @@
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>2.981786966323853</v>
+        <v>587.3197555541992</v>
       </c>
       <c r="B27" t="n">
-        <v>1422.31640625</v>
+        <v>1442.59765625</v>
       </c>
       <c r="C27" t="n">
-        <v>9.1</v>
+        <v>14.8</v>
       </c>
       <c r="D27" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="E27" t="n">
         <v>0</v>
       </c>
       <c r="F27" t="n">
-        <v>0.05086779594421387</v>
+        <v>0.3519344329833984</v>
       </c>
       <c r="G27" t="n">
-        <v>2.930916786193848</v>
+        <v>586.9678184986115</v>
       </c>
       <c r="H27" t="n">
         <v>0</v>
@@ -1148,25 +1148,25 @@
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>2.706062793731689</v>
+        <v>542.1309642791748</v>
       </c>
       <c r="B28" t="n">
-        <v>1422.3203125</v>
+        <v>1442.59765625</v>
       </c>
       <c r="C28" t="n">
-        <v>9.699999999999999</v>
+        <v>14.9</v>
       </c>
       <c r="D28" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="E28" t="n">
         <v>0</v>
       </c>
       <c r="F28" t="n">
-        <v>0.05098605155944824</v>
+        <v>0.3201277256011963</v>
       </c>
       <c r="G28" t="n">
-        <v>2.65507435798645</v>
+        <v>541.8108336925507</v>
       </c>
       <c r="H28" t="n">
         <v>0</v>
@@ -1174,25 +1174,25 @@
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>1.98659086227417</v>
+        <v>609.2033784389496</v>
       </c>
       <c r="B29" t="n">
-        <v>1422.3203125</v>
+        <v>1442.6015625</v>
       </c>
       <c r="C29" t="n">
-        <v>13.1</v>
+        <v>14.7</v>
       </c>
       <c r="D29" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="E29" t="n">
         <v>0</v>
       </c>
       <c r="F29" t="n">
-        <v>0.04817676544189453</v>
+        <v>0.3116180896759033</v>
       </c>
       <c r="G29" t="n">
-        <v>1.938410758972168</v>
+        <v>608.891758441925</v>
       </c>
       <c r="H29" t="n">
         <v>0</v>
@@ -1200,25 +1200,25 @@
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>3.365219831466675</v>
+        <v>715.6717762947083</v>
       </c>
       <c r="B30" t="n">
-        <v>1422.32421875</v>
+        <v>1443.12109375</v>
       </c>
       <c r="C30" t="n">
-        <v>15.3</v>
+        <v>14.9</v>
       </c>
       <c r="D30" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="E30" t="n">
         <v>0</v>
       </c>
       <c r="F30" t="n">
-        <v>0.04976081848144531</v>
+        <v>0.3453819751739502</v>
       </c>
       <c r="G30" t="n">
-        <v>3.315456628799438</v>
+        <v>715.3263916969299</v>
       </c>
       <c r="H30" t="n">
         <v>0</v>
@@ -1226,25 +1226,25 @@
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>4.070449829101562</v>
+        <v>539.8172943592072</v>
       </c>
       <c r="B31" t="n">
-        <v>1422.32421875</v>
+        <v>1443.125</v>
       </c>
       <c r="C31" t="n">
-        <v>9.199999999999999</v>
+        <v>14.9</v>
       </c>
       <c r="D31" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="E31" t="n">
         <v>0</v>
       </c>
       <c r="F31" t="n">
-        <v>0.04813933372497559</v>
+        <v>0.287379264831543</v>
       </c>
       <c r="G31" t="n">
-        <v>4.022308111190796</v>
+        <v>539.5299122333527</v>
       </c>
       <c r="H31" t="n">
         <v>0</v>
@@ -1252,25 +1252,25 @@
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>3.439343214035034</v>
+        <v>729.7689716815948</v>
       </c>
       <c r="B32" t="n">
-        <v>1422.32421875</v>
+        <v>1443.4453125</v>
       </c>
       <c r="C32" t="n">
-        <v>9.5</v>
+        <v>14.9</v>
       </c>
       <c r="D32" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="E32" t="n">
         <v>0</v>
       </c>
       <c r="F32" t="n">
-        <v>0.05108213424682617</v>
+        <v>0.3544979095458984</v>
       </c>
       <c r="G32" t="n">
-        <v>3.388258218765259</v>
+        <v>729.4144704341888</v>
       </c>
       <c r="H32" t="n">
         <v>0</v>
@@ -1278,25 +1278,25 @@
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>3.484983205795288</v>
+        <v>824.2940349578857</v>
       </c>
       <c r="B33" t="n">
-        <v>1422.3359375</v>
+        <v>1444.0390625</v>
       </c>
       <c r="C33" t="n">
-        <v>15.2</v>
+        <v>14.9</v>
       </c>
       <c r="D33" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="E33" t="n">
         <v>0</v>
       </c>
       <c r="F33" t="n">
-        <v>0.05068540573120117</v>
+        <v>0.4146378040313721</v>
       </c>
       <c r="G33" t="n">
-        <v>3.434294700622559</v>
+        <v>823.8793940544128</v>
       </c>
       <c r="H33" t="n">
         <v>0</v>
@@ -1304,25 +1304,25 @@
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>2.926429033279419</v>
+        <v>627.6685984134674</v>
       </c>
       <c r="B34" t="n">
-        <v>1422.33984375</v>
+        <v>1444.0390625</v>
       </c>
       <c r="C34" t="n">
-        <v>11.5</v>
+        <v>14.9</v>
       </c>
       <c r="D34" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="E34" t="n">
         <v>0</v>
       </c>
       <c r="F34" t="n">
-        <v>0.0569605827331543</v>
+        <v>0.3398356437683105</v>
       </c>
       <c r="G34" t="n">
-        <v>2.869465827941895</v>
+        <v>627.328759431839</v>
       </c>
       <c r="H34" t="n">
         <v>0</v>
@@ -1330,25 +1330,25 @@
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>2.94305944442749</v>
+        <v>684.7271406650543</v>
       </c>
       <c r="B35" t="n">
-        <v>1422.33984375</v>
+        <v>1444.0390625</v>
       </c>
       <c r="C35" t="n">
-        <v>9.199999999999999</v>
+        <v>14.9</v>
       </c>
       <c r="D35" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="E35" t="n">
         <v>0</v>
       </c>
       <c r="F35" t="n">
-        <v>0.04979109764099121</v>
+        <v>0.3410096168518066</v>
       </c>
       <c r="G35" t="n">
-        <v>2.893265962600708</v>
+        <v>684.3861281871796</v>
       </c>
       <c r="H35" t="n">
         <v>0</v>
@@ -1356,25 +1356,25 @@
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>1.753557443618774</v>
+        <v>653.0941278934479</v>
       </c>
       <c r="B36" t="n">
-        <v>1422.37109375</v>
+        <v>1444.0390625</v>
       </c>
       <c r="C36" t="n">
-        <v>9</v>
+        <v>14.8</v>
       </c>
       <c r="D36" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="E36" t="n">
         <v>0</v>
       </c>
       <c r="F36" t="n">
-        <v>0.04977202415466309</v>
+        <v>0.3627238273620605</v>
       </c>
       <c r="G36" t="n">
-        <v>1.703783273696899</v>
+        <v>652.7314004898071</v>
       </c>
       <c r="H36" t="n">
         <v>0</v>
@@ -1382,25 +1382,25 @@
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>3.355324506759644</v>
+        <v>1078.868446111679</v>
       </c>
       <c r="B37" t="n">
-        <v>1422.3984375</v>
+        <v>1444.98828125</v>
       </c>
       <c r="C37" t="n">
-        <v>10</v>
+        <v>14.9</v>
       </c>
       <c r="D37" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="E37" t="n">
         <v>0</v>
       </c>
       <c r="F37" t="n">
-        <v>0.05428695678710938</v>
+        <v>0.3251335620880127</v>
       </c>
       <c r="G37" t="n">
-        <v>3.301034927368164</v>
+        <v>1078.543310403824</v>
       </c>
       <c r="H37" t="n">
         <v>0</v>
@@ -1408,25 +1408,25 @@
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>4.005668640136719</v>
+        <v>940.9017860889435</v>
       </c>
       <c r="B38" t="n">
-        <v>1422.4296875</v>
+        <v>1445</v>
       </c>
       <c r="C38" t="n">
-        <v>15.3</v>
+        <v>14.9</v>
       </c>
       <c r="D38" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="E38" t="n">
         <v>0</v>
       </c>
       <c r="F38" t="n">
-        <v>0.04824423789978027</v>
+        <v>0.3879053592681885</v>
       </c>
       <c r="G38" t="n">
-        <v>3.957422018051147</v>
+        <v>940.5138783454895</v>
       </c>
       <c r="H38" t="n">
         <v>0</v>
@@ -1434,25 +1434,25 @@
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>3.921993255615234</v>
+        <v>922.9729022979736</v>
       </c>
       <c r="B39" t="n">
-        <v>1422.453125</v>
+        <v>1445</v>
       </c>
       <c r="C39" t="n">
-        <v>9.4</v>
+        <v>14.9</v>
       </c>
       <c r="D39" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="E39" t="n">
         <v>0</v>
       </c>
       <c r="F39" t="n">
-        <v>0.05202078819274902</v>
+        <v>0.3162760734558105</v>
       </c>
       <c r="G39" t="n">
-        <v>3.869969606399536</v>
+        <v>922.6566236019135</v>
       </c>
       <c r="H39" t="n">
         <v>0</v>
@@ -1460,25 +1460,25 @@
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>2.564812898635864</v>
+        <v>558.5937104225159</v>
       </c>
       <c r="B40" t="n">
-        <v>1422.45703125</v>
+        <v>1445.03515625</v>
       </c>
       <c r="C40" t="n">
-        <v>9.199999999999999</v>
+        <v>14.8</v>
       </c>
       <c r="D40" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="E40" t="n">
         <v>0</v>
       </c>
       <c r="F40" t="n">
-        <v>0.0503685474395752</v>
+        <v>0.3481156826019287</v>
       </c>
       <c r="G40" t="n">
-        <v>2.514441728591919</v>
+        <v>558.245591878891</v>
       </c>
       <c r="H40" t="n">
         <v>0</v>
@@ -1486,25 +1486,25 @@
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>4.765000581741333</v>
+        <v>544.0178151130676</v>
       </c>
       <c r="B41" t="n">
-        <v>1422.45703125</v>
+        <v>1445.03515625</v>
       </c>
       <c r="C41" t="n">
-        <v>14.4</v>
+        <v>14.8</v>
       </c>
       <c r="D41" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="E41" t="n">
         <v>0</v>
       </c>
       <c r="F41" t="n">
-        <v>0.04954099655151367</v>
+        <v>0.3254942893981934</v>
       </c>
       <c r="G41" t="n">
-        <v>4.715457439422607</v>
+        <v>543.6923179626465</v>
       </c>
       <c r="H41" t="n">
         <v>0</v>
@@ -1512,25 +1512,25 @@
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>2.236819982528687</v>
+        <v>515.2861828804016</v>
       </c>
       <c r="B42" t="n">
-        <v>1422.45703125</v>
+        <v>1445.03515625</v>
       </c>
       <c r="C42" t="n">
-        <v>11</v>
+        <v>14.7</v>
       </c>
       <c r="D42" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="E42" t="n">
         <v>0</v>
       </c>
       <c r="F42" t="n">
-        <v>0.04942798614501953</v>
+        <v>0.3316259384155273</v>
       </c>
       <c r="G42" t="n">
-        <v>2.187389373779297</v>
+        <v>514.9545543193817</v>
       </c>
       <c r="H42" t="n">
         <v>0</v>
@@ -1538,25 +1538,25 @@
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>4.08667516708374</v>
+        <v>758.6524956226349</v>
       </c>
       <c r="B43" t="n">
-        <v>1422.50390625</v>
+        <v>1445.03515625</v>
       </c>
       <c r="C43" t="n">
-        <v>9</v>
+        <v>14.8</v>
       </c>
       <c r="D43" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="E43" t="n">
         <v>0</v>
       </c>
       <c r="F43" t="n">
-        <v>0.04786229133605957</v>
+        <v>0.3647973537445068</v>
       </c>
       <c r="G43" t="n">
-        <v>4.03881049156189</v>
+        <v>758.2876961231232</v>
       </c>
       <c r="H43" t="n">
         <v>0</v>
@@ -1564,25 +1564,25 @@
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>3.664190769195557</v>
+        <v>562.6885273456573</v>
       </c>
       <c r="B44" t="n">
-        <v>1422.6171875</v>
+        <v>1445.03515625</v>
       </c>
       <c r="C44" t="n">
-        <v>8.9</v>
+        <v>14.7</v>
       </c>
       <c r="D44" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="E44" t="n">
         <v>0</v>
       </c>
       <c r="F44" t="n">
-        <v>0.09503722190856934</v>
+        <v>0.2901527881622314</v>
       </c>
       <c r="G44" t="n">
-        <v>3.569151163101196</v>
+        <v>562.3983726501465</v>
       </c>
       <c r="H44" t="n">
         <v>0</v>
@@ -1590,25 +1590,25 @@
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>4.24666428565979</v>
+        <v>930.8256151676178</v>
       </c>
       <c r="B45" t="n">
-        <v>1423.015625</v>
+        <v>1445.5390625</v>
       </c>
       <c r="C45" t="n">
-        <v>15.7</v>
+        <v>14.8</v>
       </c>
       <c r="D45" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="E45" t="n">
         <v>0</v>
       </c>
       <c r="F45" t="n">
-        <v>0.04938316345214844</v>
+        <v>0.3630199432373047</v>
       </c>
       <c r="G45" t="n">
-        <v>4.19727897644043</v>
+        <v>930.4625926017761</v>
       </c>
       <c r="H45" t="n">
         <v>0</v>
@@ -1616,25 +1616,25 @@
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>4.006691694259644</v>
+        <v>1153.548094749451</v>
       </c>
       <c r="B46" t="n">
-        <v>1423.0625</v>
+        <v>1445.6640625</v>
       </c>
       <c r="C46" t="n">
-        <v>9.1</v>
+        <v>14.9</v>
       </c>
       <c r="D46" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="E46" t="n">
         <v>0</v>
       </c>
       <c r="F46" t="n">
-        <v>0.05080652236938477</v>
+        <v>0.2896955013275146</v>
       </c>
       <c r="G46" t="n">
-        <v>3.955883026123047</v>
+        <v>1153.258396625519</v>
       </c>
       <c r="H46" t="n">
         <v>0</v>
@@ -1642,25 +1642,25 @@
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>3.65123987197876</v>
+        <v>815.7368252277374</v>
       </c>
       <c r="B47" t="n">
-        <v>1423.06640625</v>
+        <v>1445.6640625</v>
       </c>
       <c r="C47" t="n">
-        <v>9.300000000000001</v>
+        <v>14.8</v>
       </c>
       <c r="D47" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="E47" t="n">
         <v>0</v>
       </c>
       <c r="F47" t="n">
-        <v>0.04985165596008301</v>
+        <v>0.3509232997894287</v>
       </c>
       <c r="G47" t="n">
-        <v>3.601385831832886</v>
+        <v>815.3858995437622</v>
       </c>
       <c r="H47" t="n">
         <v>0</v>
@@ -1668,25 +1668,25 @@
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>4.871865510940552</v>
+        <v>493.434280872345</v>
       </c>
       <c r="B48" t="n">
-        <v>1423.0703125</v>
+        <v>1445.6640625</v>
       </c>
       <c r="C48" t="n">
-        <v>14.9</v>
+        <v>14.7</v>
       </c>
       <c r="D48" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="E48" t="n">
         <v>0</v>
       </c>
       <c r="F48" t="n">
-        <v>0.04800105094909668</v>
+        <v>0.3063089847564697</v>
       </c>
       <c r="G48" t="n">
-        <v>4.823861837387085</v>
+        <v>493.1279697418213</v>
       </c>
       <c r="H48" t="n">
         <v>0</v>
@@ -1694,25 +1694,25 @@
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>4.635505437850952</v>
+        <v>728.4343800544739</v>
       </c>
       <c r="B49" t="n">
-        <v>1423.07421875</v>
+        <v>1445.6640625</v>
       </c>
       <c r="C49" t="n">
-        <v>9.4</v>
+        <v>14.9</v>
       </c>
       <c r="D49" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="E49" t="n">
         <v>0</v>
       </c>
       <c r="F49" t="n">
-        <v>0.04939031600952148</v>
+        <v>0.3673627376556396</v>
       </c>
       <c r="G49" t="n">
-        <v>4.586111545562744</v>
+        <v>728.0670149326324</v>
       </c>
       <c r="H49" t="n">
         <v>0</v>
@@ -1720,25 +1720,25 @@
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>2.50710391998291</v>
+        <v>715.9503984451294</v>
       </c>
       <c r="B50" t="n">
-        <v>1423.07421875</v>
+        <v>1445.6640625</v>
       </c>
       <c r="C50" t="n">
-        <v>9.5</v>
+        <v>14.8</v>
       </c>
       <c r="D50" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="E50" t="n">
         <v>0</v>
       </c>
       <c r="F50" t="n">
-        <v>0.04818630218505859</v>
+        <v>0.3300049304962158</v>
       </c>
       <c r="G50" t="n">
-        <v>2.458915233612061</v>
+        <v>715.6203908920288</v>
       </c>
       <c r="H50" t="n">
         <v>0</v>
@@ -1746,25 +1746,25 @@
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>4.730875492095947</v>
+        <v>768.2540550231934</v>
       </c>
       <c r="B51" t="n">
-        <v>1423.078125</v>
+        <v>1445.6640625</v>
       </c>
       <c r="C51" t="n">
-        <v>14</v>
+        <v>14.8</v>
       </c>
       <c r="D51" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="E51" t="n">
         <v>0</v>
       </c>
       <c r="F51" t="n">
-        <v>0.04832935333251953</v>
+        <v>0.320411205291748</v>
       </c>
       <c r="G51" t="n">
-        <v>4.682543039321899</v>
+        <v>767.9336414337158</v>
       </c>
       <c r="H51" t="n">
         <v>0</v>
@@ -1772,25 +1772,25 @@
     </row>
     <row r="52">
       <c r="A52" t="n">
-        <v>3.884873867034912</v>
+        <v>3799.775583744049</v>
       </c>
       <c r="B52" t="n">
-        <v>1423.078125</v>
+        <v>1455.15234375</v>
       </c>
       <c r="C52" t="n">
-        <v>10.4</v>
+        <v>15.1</v>
       </c>
       <c r="D52" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="E52" t="n">
         <v>0</v>
       </c>
       <c r="F52" t="n">
-        <v>0.04909348487854004</v>
+        <v>0.3076622486114502</v>
       </c>
       <c r="G52" t="n">
-        <v>3.835777997970581</v>
+        <v>3799.46791934967</v>
       </c>
       <c r="H52" t="n">
         <v>0</v>
@@ -1798,25 +1798,25 @@
     </row>
     <row r="53">
       <c r="A53" t="n">
-        <v>4.881121873855591</v>
+        <v>1037.669524908066</v>
       </c>
       <c r="B53" t="n">
-        <v>1423.1875</v>
+        <v>1445.98828125</v>
       </c>
       <c r="C53" t="n">
-        <v>9.300000000000001</v>
+        <v>15</v>
       </c>
       <c r="D53" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="E53" t="n">
         <v>0</v>
       </c>
       <c r="F53" t="n">
-        <v>0.05055809020996094</v>
+        <v>0.3952124118804932</v>
       </c>
       <c r="G53" t="n">
-        <v>4.830561399459839</v>
+        <v>1037.274310112</v>
       </c>
       <c r="H53" t="n">
         <v>0</v>
@@ -1824,25 +1824,25 @@
     </row>
     <row r="54">
       <c r="A54" t="n">
-        <v>3.452468395233154</v>
+        <v>866.4984965324402</v>
       </c>
       <c r="B54" t="n">
-        <v>1423.19140625</v>
+        <v>1445.98828125</v>
       </c>
       <c r="C54" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D54" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="E54" t="n">
         <v>0</v>
       </c>
       <c r="F54" t="n">
-        <v>0.0521395206451416</v>
+        <v>0.3477792739868164</v>
       </c>
       <c r="G54" t="n">
-        <v>3.400325775146484</v>
+        <v>866.1507148742676</v>
       </c>
       <c r="H54" t="n">
         <v>0</v>
@@ -1850,25 +1850,25 @@
     </row>
     <row r="55">
       <c r="A55" t="n">
-        <v>4.054037570953369</v>
+        <v>719.1867294311523</v>
       </c>
       <c r="B55" t="n">
-        <v>1423.1953125</v>
+        <v>1445.98828125</v>
       </c>
       <c r="C55" t="n">
-        <v>12</v>
+        <v>14.9</v>
       </c>
       <c r="D55" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="E55" t="n">
         <v>0</v>
       </c>
       <c r="F55" t="n">
-        <v>0.05701875686645508</v>
+        <v>0.2929694652557373</v>
       </c>
       <c r="G55" t="n">
-        <v>3.997016668319702</v>
+        <v>718.8937573432922</v>
       </c>
       <c r="H55" t="n">
         <v>0</v>
@@ -1876,25 +1876,25 @@
     </row>
     <row r="56">
       <c r="A56" t="n">
-        <v>2.684615135192871</v>
+        <v>0.7618575096130371</v>
       </c>
       <c r="B56" t="n">
-        <v>1423.19921875</v>
+        <v>1440.7578125</v>
       </c>
       <c r="C56" t="n">
-        <v>9.199999999999999</v>
+        <v>9.5</v>
       </c>
       <c r="D56" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E56" t="n">
         <v>0</v>
       </c>
       <c r="F56" t="n">
-        <v>0.05046415328979492</v>
+        <v>0.7547931671142578</v>
       </c>
       <c r="G56" t="n">
-        <v>2.634148359298706</v>
+        <v>0.007060766220092773</v>
       </c>
       <c r="H56" t="n">
         <v>0</v>
@@ -1902,25 +1902,25 @@
     </row>
     <row r="57">
       <c r="A57" t="n">
-        <v>9.440521955490112</v>
+        <v>0.09327483177185059</v>
       </c>
       <c r="B57" t="n">
-        <v>1423.203125</v>
+        <v>1442.0234375</v>
       </c>
       <c r="C57" t="n">
-        <v>12.2</v>
+        <v>0.9</v>
       </c>
       <c r="D57" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E57" t="n">
         <v>0</v>
       </c>
       <c r="F57" t="n">
-        <v>0.04923439025878906</v>
+        <v>0.08502197265625</v>
       </c>
       <c r="G57" t="n">
-        <v>9.391284465789795</v>
+        <v>0.008249521255493164</v>
       </c>
       <c r="H57" t="n">
         <v>0</v>
@@ -1928,25 +1928,25 @@
     </row>
     <row r="58">
       <c r="A58" t="n">
-        <v>3.754726409912109</v>
+        <v>0.08874917030334473</v>
       </c>
       <c r="B58" t="n">
-        <v>1423.2109375</v>
+        <v>1442.10546875</v>
       </c>
       <c r="C58" t="n">
-        <v>9.199999999999999</v>
+        <v>3.6</v>
       </c>
       <c r="D58" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E58" t="n">
         <v>0</v>
       </c>
       <c r="F58" t="n">
-        <v>0.04998636245727539</v>
+        <v>0.08184504508972168</v>
       </c>
       <c r="G58" t="n">
-        <v>3.704737186431885</v>
+        <v>0.006902217864990234</v>
       </c>
       <c r="H58" t="n">
         <v>0</v>
@@ -1954,25 +1954,25 @@
     </row>
     <row r="59">
       <c r="A59" t="n">
-        <v>3.727779388427734</v>
+        <v>0.08931779861450195</v>
       </c>
       <c r="B59" t="n">
-        <v>1423.2421875</v>
+        <v>1443.35546875</v>
       </c>
       <c r="C59" t="n">
-        <v>9.4</v>
+        <v>5.8</v>
       </c>
       <c r="D59" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E59" t="n">
         <v>0</v>
       </c>
       <c r="F59" t="n">
-        <v>0.05125260353088379</v>
+        <v>0.08235979080200195</v>
       </c>
       <c r="G59" t="n">
-        <v>3.67652440071106</v>
+        <v>0.006956338882446289</v>
       </c>
       <c r="H59" t="n">
         <v>0</v>
@@ -1980,25 +1980,25 @@
     </row>
     <row r="60">
       <c r="A60" t="n">
-        <v>3.352795362472534</v>
+        <v>0.05197334289550781</v>
       </c>
       <c r="B60" t="n">
-        <v>1423.26171875</v>
+        <v>1443.515625</v>
       </c>
       <c r="C60" t="n">
-        <v>17.5</v>
+        <v>1.6</v>
       </c>
       <c r="D60" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E60" t="n">
         <v>0</v>
       </c>
       <c r="F60" t="n">
-        <v>0.05141353607177734</v>
+        <v>0.04484128952026367</v>
       </c>
       <c r="G60" t="n">
-        <v>3.301379680633545</v>
+        <v>0.007129907608032227</v>
       </c>
       <c r="H60" t="n">
         <v>0</v>
@@ -2006,25 +2006,25 @@
     </row>
     <row r="61">
       <c r="A61" t="n">
-        <v>4.365641117095947</v>
+        <v>0.09411716461181641</v>
       </c>
       <c r="B61" t="n">
-        <v>1423.26171875</v>
+        <v>1443.56640625</v>
       </c>
       <c r="C61" t="n">
-        <v>9.199999999999999</v>
+        <v>2.6</v>
       </c>
       <c r="D61" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E61" t="n">
         <v>0</v>
       </c>
       <c r="F61" t="n">
-        <v>0.05025959014892578</v>
+        <v>0.08721041679382324</v>
       </c>
       <c r="G61" t="n">
-        <v>4.315378904342651</v>
+        <v>0.006903886795043945</v>
       </c>
       <c r="H61" t="n">
         <v>0</v>
@@ -2032,25 +2032,25 @@
     </row>
     <row r="62">
       <c r="A62" t="n">
-        <v>2.33392333984375</v>
+        <v>0.09090614318847656</v>
       </c>
       <c r="B62" t="n">
-        <v>1423.26171875</v>
+        <v>1443.58203125</v>
       </c>
       <c r="C62" t="n">
-        <v>9.4</v>
+        <v>10.7</v>
       </c>
       <c r="D62" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E62" t="n">
         <v>0</v>
       </c>
       <c r="F62" t="n">
-        <v>0.04952454566955566</v>
+        <v>0.08421874046325684</v>
       </c>
       <c r="G62" t="n">
-        <v>2.284396648406982</v>
+        <v>0.006685495376586914</v>
       </c>
       <c r="H62" t="n">
         <v>0</v>
@@ -2058,25 +2058,25 @@
     </row>
     <row r="63">
       <c r="A63" t="n">
-        <v>4.375336408615112</v>
+        <v>0.05122542381286621</v>
       </c>
       <c r="B63" t="n">
-        <v>1423.26171875</v>
+        <v>1443.67578125</v>
       </c>
       <c r="C63" t="n">
-        <v>11.8</v>
+        <v>12.7</v>
       </c>
       <c r="D63" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E63" t="n">
         <v>0</v>
       </c>
       <c r="F63" t="n">
-        <v>0.04779672622680664</v>
+        <v>0.04429101943969727</v>
       </c>
       <c r="G63" t="n">
-        <v>4.327536821365356</v>
+        <v>0.006932735443115234</v>
       </c>
       <c r="H63" t="n">
         <v>0</v>
@@ -2084,25 +2084,25 @@
     </row>
     <row r="64">
       <c r="A64" t="n">
-        <v>3.580284118652344</v>
+        <v>0.04957056045532227</v>
       </c>
       <c r="B64" t="n">
-        <v>1423.26171875</v>
+        <v>1443.71875</v>
       </c>
       <c r="C64" t="n">
-        <v>14.2</v>
+        <v>13.1</v>
       </c>
       <c r="D64" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E64" t="n">
         <v>0</v>
       </c>
       <c r="F64" t="n">
-        <v>0.05049824714660645</v>
+        <v>0.04296231269836426</v>
       </c>
       <c r="G64" t="n">
-        <v>3.529783248901367</v>
+        <v>0.006605863571166992</v>
       </c>
       <c r="H64" t="n">
         <v>0</v>
@@ -2110,25 +2110,25 @@
     </row>
     <row r="65">
       <c r="A65" t="n">
-        <v>3.449615955352783</v>
+        <v>0.06311154365539551</v>
       </c>
       <c r="B65" t="n">
-        <v>1423.26171875</v>
+        <v>1443.73046875</v>
       </c>
       <c r="C65" t="n">
-        <v>9.300000000000001</v>
+        <v>11.9</v>
       </c>
       <c r="D65" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E65" t="n">
         <v>0</v>
       </c>
       <c r="F65" t="n">
-        <v>0.05204629898071289</v>
+        <v>0.05637669563293457</v>
       </c>
       <c r="G65" t="n">
-        <v>3.3975670337677</v>
+        <v>0.00673222541809082</v>
       </c>
       <c r="H65" t="n">
         <v>0</v>
@@ -2136,25 +2136,25 @@
     </row>
     <row r="66">
       <c r="A66" t="n">
-        <v>3.2605299949646</v>
+        <v>0.05215907096862793</v>
       </c>
       <c r="B66" t="n">
-        <v>1423.27734375</v>
+        <v>1443.8359375</v>
       </c>
       <c r="C66" t="n">
-        <v>9.1</v>
+        <v>20.9</v>
       </c>
       <c r="D66" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E66" t="n">
         <v>0</v>
       </c>
       <c r="F66" t="n">
-        <v>0.04822158813476562</v>
+        <v>0.04479098320007324</v>
       </c>
       <c r="G66" t="n">
-        <v>3.212305307388306</v>
+        <v>0.007365703582763672</v>
       </c>
       <c r="H66" t="n">
         <v>0</v>
@@ -2162,25 +2162,25 @@
     </row>
     <row r="67">
       <c r="A67" t="n">
-        <v>4.323662519454956</v>
+        <v>0.05128598213195801</v>
       </c>
       <c r="B67" t="n">
-        <v>1423.34765625</v>
+        <v>1443.92578125</v>
       </c>
       <c r="C67" t="n">
-        <v>15.2</v>
+        <v>14.3</v>
       </c>
       <c r="D67" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E67" t="n">
         <v>0</v>
       </c>
       <c r="F67" t="n">
-        <v>0.04805970191955566</v>
+        <v>0.04441928863525391</v>
       </c>
       <c r="G67" t="n">
-        <v>4.275600671768188</v>
+        <v>0.006864070892333984</v>
       </c>
       <c r="H67" t="n">
         <v>0</v>
@@ -2188,25 +2188,25 @@
     </row>
     <row r="68">
       <c r="A68" t="n">
-        <v>7.325037479400635</v>
+        <v>0.05210041999816895</v>
       </c>
       <c r="B68" t="n">
-        <v>1423.37109375</v>
+        <v>1444.125</v>
       </c>
       <c r="C68" t="n">
-        <v>9.300000000000001</v>
+        <v>5.6</v>
       </c>
       <c r="D68" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E68" t="n">
         <v>0</v>
       </c>
       <c r="F68" t="n">
-        <v>0.05088114738464355</v>
+        <v>0.04439258575439453</v>
       </c>
       <c r="G68" t="n">
-        <v>7.274153470993042</v>
+        <v>0.007705926895141602</v>
       </c>
       <c r="H68" t="n">
         <v>0</v>

</xml_diff>